<commit_message>
Added week 1 stats
</commit_message>
<xml_diff>
--- a/game-stats/Week1_Pali-Gliders_vs_Good-Guys.xlsx
+++ b/game-stats/Week1_Pali-Gliders_vs_Good-Guys.xlsx
@@ -522,20 +522,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,40 +562,70 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Pass Comp</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Pass Att</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>Pass YDs</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Pass TDs</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>INTs</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Rush Att</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Rush YDs</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Rec YDs</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>TDs</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>INTs</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Def INTs</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>PBU</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Sacks</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Flag Pulls</t>
         </is>
@@ -633,6 +669,24 @@
       <c r="K2" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -672,6 +726,24 @@
       <c r="K3" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -711,6 +783,24 @@
       <c r="K4" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -750,6 +840,24 @@
       <c r="K5" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -789,6 +897,24 @@
       <c r="K6" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -828,6 +954,24 @@
       <c r="K7" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -867,6 +1011,24 @@
       <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -906,6 +1068,24 @@
       <c r="K9" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -945,6 +1125,24 @@
       <c r="K10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -982,6 +1180,24 @@
         <v>0</v>
       </c>
       <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1023,6 +1239,24 @@
       <c r="K12" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1062,6 +1296,24 @@
       <c r="K13" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1101,6 +1353,24 @@
       <c r="K14" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1138,6 +1408,24 @@
         <v>0</v>
       </c>
       <c r="K15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1152,20 +1440,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1186,40 +1480,70 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Pass Comp</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Pass Att</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>Pass YDs</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Pass TDs</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>INTs</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Rush Att</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Rush YDs</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Rec YDs</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>TDs</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>INTs</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Def INTs</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>PBU</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Sacks</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Flag Pulls</t>
         </is>
@@ -1263,6 +1587,24 @@
       <c r="K2" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -1302,6 +1644,24 @@
       <c r="K3" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -1341,6 +1701,24 @@
       <c r="K4" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1380,6 +1758,24 @@
       <c r="K5" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -1419,6 +1815,24 @@
       <c r="K6" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1458,6 +1872,24 @@
       <c r="K7" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1497,6 +1929,24 @@
       <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1536,6 +1986,24 @@
       <c r="K9" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1573,6 +2041,24 @@
         <v>0</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>